<commit_message>
updated simulation with parameter calibration (pre-run)
</commit_message>
<xml_diff>
--- a/analysis/2026_05_05_parameters.xlsx
+++ b/analysis/2026_05_05_parameters.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="141" documentId="11_A2545D69FD1DC248E0D100DFBCDD0C6123C0B3C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D6D3D3D3-BBDD-C54B-B146-4468C8D4DFB4}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="18280" yWindow="29460" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1 Pre-existing Infection" sheetId="1" r:id="rId1"/>
@@ -572,11 +572,11 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -586,7 +586,7 @@
     <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
@@ -608,6 +608,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>